<commit_message>
preprocessed info for statistic analysis
</commit_message>
<xml_diff>
--- a/data/department_schedules_finals/İnşaat Mühendisliği.xlsx
+++ b/data/department_schedules_finals/İnşaat Mühendisliği.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\department_schedules_finals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{0E0A3EA1-C2E2-4B1F-84AC-00B429DE38D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0125CA14-4C83-45E6-AF12-F93E24920358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3800" yWindow="3800" windowWidth="28920" windowHeight="10250" xr2:uid="{91744B99-4786-4948-8AC9-0C0F2BECAA6A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{91744B99-4786-4948-8AC9-0C0F2BECAA6A}"/>
   </bookViews>
   <sheets>
     <sheet name="Filled_Exam_Schedule" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Year:</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t>MAT 162</t>
-  </si>
-  <si>
-    <t>JEO 308</t>
   </si>
   <si>
     <t>İNM 104</t>
@@ -706,8 +703,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C5046FB1-8390-49B0-AA15-6AA3F4A2AFF1}" name="Table1" displayName="Table1" ref="A1:D35" totalsRowShown="0">
-  <autoFilter ref="A1:D35" xr:uid="{C5046FB1-8390-49B0-AA15-6AA3F4A2AFF1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C5046FB1-8390-49B0-AA15-6AA3F4A2AFF1}" name="Table1" displayName="Table1" ref="A1:D34" totalsRowShown="0">
+  <autoFilter ref="A1:D34" xr:uid="{C5046FB1-8390-49B0-AA15-6AA3F4A2AFF1}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DB671DE9-90D2-4C2F-8769-14A7073BEBFA}" name="Year:"/>
     <tableColumn id="2" xr3:uid="{7494E69D-90F9-44A0-9128-0CAACE54C220}" name="Course ID"/>
@@ -1035,7 +1032,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF810464-3772-4692-AFA3-F8000F5D7FFA}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.7265625" customWidth="1"/>
@@ -1060,7 +1057,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1">
         <v>8</v>
@@ -1074,7 +1071,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1">
         <v>2</v>
@@ -1088,7 +1085,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1">
         <v>5</v>
@@ -1116,7 +1113,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1">
         <v>7</v>
@@ -1144,7 +1141,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="1">
         <v>1</v>
@@ -1158,7 +1155,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
@@ -1172,7 +1169,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
@@ -1186,7 +1183,7 @@
         <v>2</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11" s="2">
         <v>3</v>
@@ -1200,7 +1197,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" s="2">
         <v>3</v>
@@ -1214,7 +1211,7 @@
         <v>2</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13" s="2">
         <v>5</v>
@@ -1228,7 +1225,7 @@
         <v>2</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2">
         <v>6</v>
@@ -1242,7 +1239,7 @@
         <v>2</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C15" s="2">
         <v>7</v>
@@ -1256,7 +1253,7 @@
         <v>3</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C16" s="3">
         <v>7</v>
@@ -1270,7 +1267,7 @@
         <v>3</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17" s="3">
         <v>6</v>
@@ -1284,7 +1281,7 @@
         <v>3</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" s="3">
         <v>4</v>
@@ -1298,7 +1295,7 @@
         <v>3</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C19" s="3">
         <v>4</v>
@@ -1312,7 +1309,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C20" s="3">
         <v>8</v>
@@ -1326,7 +1323,7 @@
         <v>3</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" s="3">
         <v>1</v>
@@ -1340,7 +1337,7 @@
         <v>3</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C22" s="3">
         <v>8</v>
@@ -1354,7 +1351,7 @@
         <v>3</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C23" s="3">
         <v>7</v>
@@ -1368,7 +1365,7 @@
         <v>3</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="C24" s="3">
         <v>5</v>
@@ -1378,17 +1375,17 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="3">
-        <v>3</v>
-      </c>
-      <c r="B25" s="3" t="s">
+      <c r="A25" s="4">
+        <v>4</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="3">
-        <v>5</v>
-      </c>
-      <c r="D25" s="3">
-        <v>2</v>
+      <c r="C25" s="4">
+        <v>7</v>
+      </c>
+      <c r="D25" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -1399,10 +1396,10 @@
         <v>28</v>
       </c>
       <c r="C26" s="4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D26" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
@@ -1413,7 +1410,7 @@
         <v>29</v>
       </c>
       <c r="C27" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="4">
         <v>2</v>
@@ -1427,10 +1424,10 @@
         <v>30</v>
       </c>
       <c r="C28" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -1441,7 +1438,7 @@
         <v>31</v>
       </c>
       <c r="C29" s="4">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D29" s="4">
         <v>1</v>
@@ -1455,7 +1452,7 @@
         <v>32</v>
       </c>
       <c r="C30" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D30" s="4">
         <v>1</v>
@@ -1469,7 +1466,7 @@
         <v>33</v>
       </c>
       <c r="C31" s="4">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D31" s="4">
         <v>1</v>
@@ -1483,7 +1480,7 @@
         <v>34</v>
       </c>
       <c r="C32" s="4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D32" s="4">
         <v>1</v>
@@ -1497,7 +1494,7 @@
         <v>35</v>
       </c>
       <c r="C33" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33" s="4">
         <v>1</v>
@@ -1511,23 +1508,9 @@
         <v>36</v>
       </c>
       <c r="C34" s="4">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D34" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="4">
-        <v>4</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C35" s="4">
-        <v>8</v>
-      </c>
-      <c r="D35" s="4">
         <v>1</v>
       </c>
     </row>

</xml_diff>